<commit_message>
Small code refinements and update predictions 17.06.2026
</commit_message>
<xml_diff>
--- a/processed_data_during_wm/processed_data_long.xlsx
+++ b/processed_data_during_wm/processed_data_long.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="56">
   <si>
     <t>Team</t>
   </si>
@@ -543,7 +543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H145"/>
+  <dimension ref="A1:H193"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -4316,6 +4316,1254 @@
         <v>0.0026</v>
       </c>
     </row>
+    <row r="146" spans="1:8">
+      <c r="A146" t="s">
+        <v>9</v>
+      </c>
+      <c r="B146" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C146">
+        <v>7</v>
+      </c>
+      <c r="D146">
+        <v>4.9671</v>
+      </c>
+      <c r="E146">
+        <v>0.168128</v>
+      </c>
+      <c r="F146">
+        <v>16.8128</v>
+      </c>
+      <c r="G146">
+        <v>0.181375</v>
+      </c>
+      <c r="H146">
+        <v>18.1375</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8">
+      <c r="A147" t="s">
+        <v>8</v>
+      </c>
+      <c r="B147" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C147">
+        <v>7</v>
+      </c>
+      <c r="D147">
+        <v>6.5114</v>
+      </c>
+      <c r="E147">
+        <v>0.128254</v>
+      </c>
+      <c r="F147">
+        <v>12.8254</v>
+      </c>
+      <c r="G147">
+        <v>0.13761</v>
+      </c>
+      <c r="H147">
+        <v>13.761</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8">
+      <c r="A148" t="s">
+        <v>10</v>
+      </c>
+      <c r="B148" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C148">
+        <v>7</v>
+      </c>
+      <c r="D148">
+        <v>8.334300000000001</v>
+      </c>
+      <c r="E148">
+        <v>0.100202</v>
+      </c>
+      <c r="F148">
+        <v>10.0202</v>
+      </c>
+      <c r="G148">
+        <v>0.106826</v>
+      </c>
+      <c r="H148">
+        <v>10.6826</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8">
+      <c r="A149" t="s">
+        <v>11</v>
+      </c>
+      <c r="B149" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C149">
+        <v>7</v>
+      </c>
+      <c r="D149">
+        <v>8.617100000000001</v>
+      </c>
+      <c r="E149">
+        <v>0.096913</v>
+      </c>
+      <c r="F149">
+        <v>9.6913</v>
+      </c>
+      <c r="G149">
+        <v>0.103217</v>
+      </c>
+      <c r="H149">
+        <v>10.3217</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8">
+      <c r="A150" t="s">
+        <v>13</v>
+      </c>
+      <c r="B150" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C150">
+        <v>7</v>
+      </c>
+      <c r="D150">
+        <v>9.4</v>
+      </c>
+      <c r="E150">
+        <v>0.088842</v>
+      </c>
+      <c r="F150">
+        <v>8.8842</v>
+      </c>
+      <c r="G150">
+        <v>0.094361</v>
+      </c>
+      <c r="H150">
+        <v>9.4361</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8">
+      <c r="A151" t="s">
+        <v>12</v>
+      </c>
+      <c r="B151" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C151">
+        <v>7</v>
+      </c>
+      <c r="D151">
+        <v>11.3857</v>
+      </c>
+      <c r="E151">
+        <v>0.073348</v>
+      </c>
+      <c r="F151">
+        <v>7.3348</v>
+      </c>
+      <c r="G151">
+        <v>0.077362</v>
+      </c>
+      <c r="H151">
+        <v>7.7362</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8">
+      <c r="A152" t="s">
+        <v>14</v>
+      </c>
+      <c r="B152" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C152">
+        <v>7</v>
+      </c>
+      <c r="D152">
+        <v>14.6714</v>
+      </c>
+      <c r="E152">
+        <v>0.056921</v>
+      </c>
+      <c r="F152">
+        <v>5.6921</v>
+      </c>
+      <c r="G152">
+        <v>0.059348</v>
+      </c>
+      <c r="H152">
+        <v>5.9348</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8">
+      <c r="A153" t="s">
+        <v>15</v>
+      </c>
+      <c r="B153" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C153">
+        <v>7</v>
+      </c>
+      <c r="D153">
+        <v>20.1429</v>
+      </c>
+      <c r="E153">
+        <v>0.04146</v>
+      </c>
+      <c r="F153">
+        <v>4.146</v>
+      </c>
+      <c r="G153">
+        <v>0.042405</v>
+      </c>
+      <c r="H153">
+        <v>4.2405</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8">
+      <c r="A154" t="s">
+        <v>16</v>
+      </c>
+      <c r="B154" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C154">
+        <v>7</v>
+      </c>
+      <c r="D154">
+        <v>30.4286</v>
+      </c>
+      <c r="E154">
+        <v>0.027445</v>
+      </c>
+      <c r="F154">
+        <v>2.7445</v>
+      </c>
+      <c r="G154">
+        <v>0.027078</v>
+      </c>
+      <c r="H154">
+        <v>2.7078</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8">
+      <c r="A155" t="s">
+        <v>19</v>
+      </c>
+      <c r="B155" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C155">
+        <v>7</v>
+      </c>
+      <c r="D155">
+        <v>37.7143</v>
+      </c>
+      <c r="E155">
+        <v>0.022143</v>
+      </c>
+      <c r="F155">
+        <v>2.2143</v>
+      </c>
+      <c r="G155">
+        <v>0.021298</v>
+      </c>
+      <c r="H155">
+        <v>2.1298</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8">
+      <c r="A156" t="s">
+        <v>21</v>
+      </c>
+      <c r="B156" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C156">
+        <v>7</v>
+      </c>
+      <c r="D156">
+        <v>41.1429</v>
+      </c>
+      <c r="E156">
+        <v>0.020298</v>
+      </c>
+      <c r="F156">
+        <v>2.0298</v>
+      </c>
+      <c r="G156">
+        <v>0.019292</v>
+      </c>
+      <c r="H156">
+        <v>1.9292</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8">
+      <c r="A157" t="s">
+        <v>17</v>
+      </c>
+      <c r="B157" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C157">
+        <v>7</v>
+      </c>
+      <c r="D157">
+        <v>42</v>
+      </c>
+      <c r="E157">
+        <v>0.019884</v>
+      </c>
+      <c r="F157">
+        <v>1.9884</v>
+      </c>
+      <c r="G157">
+        <v>0.018842</v>
+      </c>
+      <c r="H157">
+        <v>1.8842</v>
+      </c>
+    </row>
+    <row r="158" spans="1:8">
+      <c r="A158" t="s">
+        <v>18</v>
+      </c>
+      <c r="B158" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C158">
+        <v>7</v>
+      </c>
+      <c r="D158">
+        <v>50.4286</v>
+      </c>
+      <c r="E158">
+        <v>0.01656</v>
+      </c>
+      <c r="F158">
+        <v>1.656</v>
+      </c>
+      <c r="G158">
+        <v>0.01524</v>
+      </c>
+      <c r="H158">
+        <v>1.524</v>
+      </c>
+    </row>
+    <row r="159" spans="1:8">
+      <c r="A159" t="s">
+        <v>20</v>
+      </c>
+      <c r="B159" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C159">
+        <v>7</v>
+      </c>
+      <c r="D159">
+        <v>51.2857</v>
+      </c>
+      <c r="E159">
+        <v>0.016284</v>
+      </c>
+      <c r="F159">
+        <v>1.6284</v>
+      </c>
+      <c r="G159">
+        <v>0.014941</v>
+      </c>
+      <c r="H159">
+        <v>1.4941</v>
+      </c>
+    </row>
+    <row r="160" spans="1:8">
+      <c r="A160" t="s">
+        <v>22</v>
+      </c>
+      <c r="B160" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C160">
+        <v>7</v>
+      </c>
+      <c r="D160">
+        <v>57.8571</v>
+      </c>
+      <c r="E160">
+        <v>0.014434</v>
+      </c>
+      <c r="F160">
+        <v>1.4434</v>
+      </c>
+      <c r="G160">
+        <v>0.012947</v>
+      </c>
+      <c r="H160">
+        <v>1.2947</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8">
+      <c r="A161" t="s">
+        <v>23</v>
+      </c>
+      <c r="B161" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C161">
+        <v>7</v>
+      </c>
+      <c r="D161">
+        <v>83</v>
+      </c>
+      <c r="E161">
+        <v>0.010062</v>
+      </c>
+      <c r="F161">
+        <v>1.0062</v>
+      </c>
+      <c r="G161">
+        <v>0.008283</v>
+      </c>
+      <c r="H161">
+        <v>0.8283</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8">
+      <c r="A162" t="s">
+        <v>24</v>
+      </c>
+      <c r="B162" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C162">
+        <v>7</v>
+      </c>
+      <c r="D162">
+        <v>87.71429999999999</v>
+      </c>
+      <c r="E162">
+        <v>0.009521</v>
+      </c>
+      <c r="F162">
+        <v>0.9520999999999999</v>
+      </c>
+      <c r="G162">
+        <v>0.007715</v>
+      </c>
+      <c r="H162">
+        <v>0.7715</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8">
+      <c r="A163" t="s">
+        <v>26</v>
+      </c>
+      <c r="B163" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C163">
+        <v>7</v>
+      </c>
+      <c r="D163">
+        <v>92.4286</v>
+      </c>
+      <c r="E163">
+        <v>0.009035</v>
+      </c>
+      <c r="F163">
+        <v>0.9035</v>
+      </c>
+      <c r="G163">
+        <v>0.007206</v>
+      </c>
+      <c r="H163">
+        <v>0.7206</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8">
+      <c r="A164" t="s">
+        <v>29</v>
+      </c>
+      <c r="B164" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C164">
+        <v>7</v>
+      </c>
+      <c r="D164">
+        <v>105.8571</v>
+      </c>
+      <c r="E164">
+        <v>0.007889</v>
+      </c>
+      <c r="F164">
+        <v>0.7889</v>
+      </c>
+      <c r="G164">
+        <v>0.006018</v>
+      </c>
+      <c r="H164">
+        <v>0.6018</v>
+      </c>
+    </row>
+    <row r="165" spans="1:8">
+      <c r="A165" t="s">
+        <v>28</v>
+      </c>
+      <c r="B165" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C165">
+        <v>7</v>
+      </c>
+      <c r="D165">
+        <v>119.5714</v>
+      </c>
+      <c r="E165">
+        <v>0.006984</v>
+      </c>
+      <c r="F165">
+        <v>0.6984</v>
+      </c>
+      <c r="G165">
+        <v>0.005094</v>
+      </c>
+      <c r="H165">
+        <v>0.5094</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8">
+      <c r="A166" t="s">
+        <v>40</v>
+      </c>
+      <c r="B166" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C166">
+        <v>7</v>
+      </c>
+      <c r="D166">
+        <v>123.1429</v>
+      </c>
+      <c r="E166">
+        <v>0.006782</v>
+      </c>
+      <c r="F166">
+        <v>0.6782</v>
+      </c>
+      <c r="G166">
+        <v>0.00489</v>
+      </c>
+      <c r="H166">
+        <v>0.489</v>
+      </c>
+    </row>
+    <row r="167" spans="1:8">
+      <c r="A167" t="s">
+        <v>27</v>
+      </c>
+      <c r="B167" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C167">
+        <v>7</v>
+      </c>
+      <c r="D167">
+        <v>135.1429</v>
+      </c>
+      <c r="E167">
+        <v>0.006179</v>
+      </c>
+      <c r="F167">
+        <v>0.6179</v>
+      </c>
+      <c r="G167">
+        <v>0.004287</v>
+      </c>
+      <c r="H167">
+        <v>0.4287</v>
+      </c>
+    </row>
+    <row r="168" spans="1:8">
+      <c r="A168" t="s">
+        <v>30</v>
+      </c>
+      <c r="B168" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C168">
+        <v>7</v>
+      </c>
+      <c r="D168">
+        <v>135.1429</v>
+      </c>
+      <c r="E168">
+        <v>0.006179</v>
+      </c>
+      <c r="F168">
+        <v>0.6179</v>
+      </c>
+      <c r="G168">
+        <v>0.004287</v>
+      </c>
+      <c r="H168">
+        <v>0.4287</v>
+      </c>
+    </row>
+    <row r="169" spans="1:8">
+      <c r="A169" t="s">
+        <v>34</v>
+      </c>
+      <c r="B169" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C169">
+        <v>7</v>
+      </c>
+      <c r="D169">
+        <v>143</v>
+      </c>
+      <c r="E169">
+        <v>0.00584</v>
+      </c>
+      <c r="F169">
+        <v>0.584</v>
+      </c>
+      <c r="G169">
+        <v>0.003953</v>
+      </c>
+      <c r="H169">
+        <v>0.3953</v>
+      </c>
+    </row>
+    <row r="170" spans="1:8">
+      <c r="A170" t="s">
+        <v>25</v>
+      </c>
+      <c r="B170" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C170">
+        <v>7</v>
+      </c>
+      <c r="D170">
+        <v>145.8571</v>
+      </c>
+      <c r="E170">
+        <v>0.005726</v>
+      </c>
+      <c r="F170">
+        <v>0.5726</v>
+      </c>
+      <c r="G170">
+        <v>0.003841</v>
+      </c>
+      <c r="H170">
+        <v>0.3841</v>
+      </c>
+    </row>
+    <row r="171" spans="1:8">
+      <c r="A171" t="s">
+        <v>31</v>
+      </c>
+      <c r="B171" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C171">
+        <v>7</v>
+      </c>
+      <c r="D171">
+        <v>197.4286</v>
+      </c>
+      <c r="E171">
+        <v>0.00423</v>
+      </c>
+      <c r="F171">
+        <v>0.423</v>
+      </c>
+      <c r="G171">
+        <v>0.002429</v>
+      </c>
+      <c r="H171">
+        <v>0.2429</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8">
+      <c r="A172" t="s">
+        <v>33</v>
+      </c>
+      <c r="B172" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C172">
+        <v>7</v>
+      </c>
+      <c r="D172">
+        <v>216.7143</v>
+      </c>
+      <c r="E172">
+        <v>0.003854</v>
+      </c>
+      <c r="F172">
+        <v>0.3854</v>
+      </c>
+      <c r="G172">
+        <v>0.002095</v>
+      </c>
+      <c r="H172">
+        <v>0.2095</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8">
+      <c r="A173" t="s">
+        <v>39</v>
+      </c>
+      <c r="B173" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C173">
+        <v>7</v>
+      </c>
+      <c r="D173">
+        <v>234</v>
+      </c>
+      <c r="E173">
+        <v>0.003569</v>
+      </c>
+      <c r="F173">
+        <v>0.3569</v>
+      </c>
+      <c r="G173">
+        <v>0.00185</v>
+      </c>
+      <c r="H173">
+        <v>0.185</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8">
+      <c r="A174" t="s">
+        <v>36</v>
+      </c>
+      <c r="B174" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C174">
+        <v>7</v>
+      </c>
+      <c r="D174">
+        <v>283.7143</v>
+      </c>
+      <c r="E174">
+        <v>0.002944</v>
+      </c>
+      <c r="F174">
+        <v>0.2944</v>
+      </c>
+      <c r="G174">
+        <v>0.001341</v>
+      </c>
+      <c r="H174">
+        <v>0.1341</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8">
+      <c r="A175" t="s">
+        <v>38</v>
+      </c>
+      <c r="B175" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C175">
+        <v>7</v>
+      </c>
+      <c r="D175">
+        <v>390.7143</v>
+      </c>
+      <c r="E175">
+        <v>0.002137</v>
+      </c>
+      <c r="F175">
+        <v>0.2137</v>
+      </c>
+      <c r="G175">
+        <v>0.000764</v>
+      </c>
+      <c r="H175">
+        <v>0.0764</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8">
+      <c r="A176" t="s">
+        <v>37</v>
+      </c>
+      <c r="B176" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C176">
+        <v>7</v>
+      </c>
+      <c r="D176">
+        <v>474.5714</v>
+      </c>
+      <c r="E176">
+        <v>0.00176</v>
+      </c>
+      <c r="F176">
+        <v>0.176</v>
+      </c>
+      <c r="G176">
+        <v>0.000535</v>
+      </c>
+      <c r="H176">
+        <v>0.0535</v>
+      </c>
+    </row>
+    <row r="177" spans="1:8">
+      <c r="A177" t="s">
+        <v>32</v>
+      </c>
+      <c r="B177" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C177">
+        <v>7</v>
+      </c>
+      <c r="D177">
+        <v>490.7143</v>
+      </c>
+      <c r="E177">
+        <v>0.001702</v>
+      </c>
+      <c r="F177">
+        <v>0.1702</v>
+      </c>
+      <c r="G177">
+        <v>0.000502</v>
+      </c>
+      <c r="H177">
+        <v>0.0502</v>
+      </c>
+    </row>
+    <row r="178" spans="1:8">
+      <c r="A178" t="s">
+        <v>35</v>
+      </c>
+      <c r="B178" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C178">
+        <v>7</v>
+      </c>
+      <c r="D178">
+        <v>497.8571</v>
+      </c>
+      <c r="E178">
+        <v>0.001677</v>
+      </c>
+      <c r="F178">
+        <v>0.1677</v>
+      </c>
+      <c r="G178">
+        <v>0.000489</v>
+      </c>
+      <c r="H178">
+        <v>0.0489</v>
+      </c>
+    </row>
+    <row r="179" spans="1:8">
+      <c r="A179" t="s">
+        <v>41</v>
+      </c>
+      <c r="B179" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C179">
+        <v>7</v>
+      </c>
+      <c r="D179">
+        <v>502.4286</v>
+      </c>
+      <c r="E179">
+        <v>0.001662</v>
+      </c>
+      <c r="F179">
+        <v>0.1662</v>
+      </c>
+      <c r="G179">
+        <v>0.000481</v>
+      </c>
+      <c r="H179">
+        <v>0.0481</v>
+      </c>
+    </row>
+    <row r="180" spans="1:8">
+      <c r="A180" t="s">
+        <v>42</v>
+      </c>
+      <c r="B180" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C180">
+        <v>7</v>
+      </c>
+      <c r="D180">
+        <v>612.1429000000001</v>
+      </c>
+      <c r="E180">
+        <v>0.001364</v>
+      </c>
+      <c r="F180">
+        <v>0.1364</v>
+      </c>
+      <c r="G180">
+        <v>0.000331</v>
+      </c>
+      <c r="H180">
+        <v>0.0331</v>
+      </c>
+    </row>
+    <row r="181" spans="1:8">
+      <c r="A181" t="s">
+        <v>44</v>
+      </c>
+      <c r="B181" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C181">
+        <v>7</v>
+      </c>
+      <c r="D181">
+        <v>747.8570999999999</v>
+      </c>
+      <c r="E181">
+        <v>0.001117</v>
+      </c>
+      <c r="F181">
+        <v>0.1117</v>
+      </c>
+      <c r="G181">
+        <v>0.000225</v>
+      </c>
+      <c r="H181">
+        <v>0.0225</v>
+      </c>
+    </row>
+    <row r="182" spans="1:8">
+      <c r="A182" t="s">
+        <v>45</v>
+      </c>
+      <c r="B182" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C182">
+        <v>7</v>
+      </c>
+      <c r="D182">
+        <v>783.5714</v>
+      </c>
+      <c r="E182">
+        <v>0.001066</v>
+      </c>
+      <c r="F182">
+        <v>0.1066</v>
+      </c>
+      <c r="G182">
+        <v>0.000206</v>
+      </c>
+      <c r="H182">
+        <v>0.0206</v>
+      </c>
+    </row>
+    <row r="183" spans="1:8">
+      <c r="A183" t="s">
+        <v>49</v>
+      </c>
+      <c r="B183" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C183">
+        <v>7</v>
+      </c>
+      <c r="D183">
+        <v>819.2857</v>
+      </c>
+      <c r="E183">
+        <v>0.001019</v>
+      </c>
+      <c r="F183">
+        <v>0.1019</v>
+      </c>
+      <c r="G183">
+        <v>0.000189</v>
+      </c>
+      <c r="H183">
+        <v>0.0189</v>
+      </c>
+    </row>
+    <row r="184" spans="1:8">
+      <c r="A184" t="s">
+        <v>43</v>
+      </c>
+      <c r="B184" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C184">
+        <v>7</v>
+      </c>
+      <c r="D184">
+        <v>926.4286</v>
+      </c>
+      <c r="E184">
+        <v>0.000901</v>
+      </c>
+      <c r="F184">
+        <v>0.0901</v>
+      </c>
+      <c r="G184">
+        <v>0.000148</v>
+      </c>
+      <c r="H184">
+        <v>0.0148</v>
+      </c>
+    </row>
+    <row r="185" spans="1:8">
+      <c r="A185" t="s">
+        <v>52</v>
+      </c>
+      <c r="B185" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C185">
+        <v>7</v>
+      </c>
+      <c r="D185">
+        <v>1069.2857</v>
+      </c>
+      <c r="E185">
+        <v>0.000781</v>
+      </c>
+      <c r="F185">
+        <v>0.0781</v>
+      </c>
+      <c r="G185">
+        <v>0.000112</v>
+      </c>
+      <c r="H185">
+        <v>0.0112</v>
+      </c>
+    </row>
+    <row r="186" spans="1:8">
+      <c r="A186" t="s">
+        <v>47</v>
+      </c>
+      <c r="B186" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C186">
+        <v>7</v>
+      </c>
+      <c r="D186">
+        <v>1069.2857</v>
+      </c>
+      <c r="E186">
+        <v>0.000781</v>
+      </c>
+      <c r="F186">
+        <v>0.0781</v>
+      </c>
+      <c r="G186">
+        <v>0.000112</v>
+      </c>
+      <c r="H186">
+        <v>0.0112</v>
+      </c>
+    </row>
+    <row r="187" spans="1:8">
+      <c r="A187" t="s">
+        <v>46</v>
+      </c>
+      <c r="B187" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C187">
+        <v>7</v>
+      </c>
+      <c r="D187">
+        <v>1176.4286</v>
+      </c>
+      <c r="E187">
+        <v>0.00071</v>
+      </c>
+      <c r="F187">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="G187">
+        <v>9.3E-05</v>
+      </c>
+      <c r="H187">
+        <v>0.009299999999999999</v>
+      </c>
+    </row>
+    <row r="188" spans="1:8">
+      <c r="A188" t="s">
+        <v>48</v>
+      </c>
+      <c r="B188" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C188">
+        <v>7</v>
+      </c>
+      <c r="D188">
+        <v>1197.8571</v>
+      </c>
+      <c r="E188">
+        <v>0.000697</v>
+      </c>
+      <c r="F188">
+        <v>0.0697</v>
+      </c>
+      <c r="G188">
+        <v>9.000000000000001E-05</v>
+      </c>
+      <c r="H188">
+        <v>0.008999999999999999</v>
+      </c>
+    </row>
+    <row r="189" spans="1:8">
+      <c r="A189" t="s">
+        <v>50</v>
+      </c>
+      <c r="B189" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C189">
+        <v>7</v>
+      </c>
+      <c r="D189">
+        <v>1197.8571</v>
+      </c>
+      <c r="E189">
+        <v>0.000697</v>
+      </c>
+      <c r="F189">
+        <v>0.0697</v>
+      </c>
+      <c r="G189">
+        <v>9.000000000000001E-05</v>
+      </c>
+      <c r="H189">
+        <v>0.008999999999999999</v>
+      </c>
+    </row>
+    <row r="190" spans="1:8">
+      <c r="A190" t="s">
+        <v>51</v>
+      </c>
+      <c r="B190" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C190">
+        <v>7</v>
+      </c>
+      <c r="D190">
+        <v>1197.8571</v>
+      </c>
+      <c r="E190">
+        <v>0.000697</v>
+      </c>
+      <c r="F190">
+        <v>0.0697</v>
+      </c>
+      <c r="G190">
+        <v>9.000000000000001E-05</v>
+      </c>
+      <c r="H190">
+        <v>0.008999999999999999</v>
+      </c>
+    </row>
+    <row r="191" spans="1:8">
+      <c r="A191" t="s">
+        <v>53</v>
+      </c>
+      <c r="B191" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C191">
+        <v>7</v>
+      </c>
+      <c r="D191">
+        <v>1497.8571</v>
+      </c>
+      <c r="E191">
+        <v>0.000558</v>
+      </c>
+      <c r="F191">
+        <v>0.0558</v>
+      </c>
+      <c r="G191">
+        <v>5.8E-05</v>
+      </c>
+      <c r="H191">
+        <v>0.0058</v>
+      </c>
+    </row>
+    <row r="192" spans="1:8">
+      <c r="A192" t="s">
+        <v>55</v>
+      </c>
+      <c r="B192" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C192">
+        <v>7</v>
+      </c>
+      <c r="D192">
+        <v>2033.5714</v>
+      </c>
+      <c r="E192">
+        <v>0.000411</v>
+      </c>
+      <c r="F192">
+        <v>0.0411</v>
+      </c>
+      <c r="G192">
+        <v>3.1E-05</v>
+      </c>
+      <c r="H192">
+        <v>0.0031</v>
+      </c>
+    </row>
+    <row r="193" spans="1:8">
+      <c r="A193" t="s">
+        <v>54</v>
+      </c>
+      <c r="B193" s="2">
+        <v>46190</v>
+      </c>
+      <c r="C193">
+        <v>7</v>
+      </c>
+      <c r="D193">
+        <v>2355</v>
+      </c>
+      <c r="E193">
+        <v>0.000355</v>
+      </c>
+      <c r="F193">
+        <v>0.0355</v>
+      </c>
+      <c r="G193">
+        <v>2.3E-05</v>
+      </c>
+      <c r="H193">
+        <v>0.0023</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixing bugs and update prediction 26.06.2026
</commit_message>
<xml_diff>
--- a/processed_data_during_wm/processed_data_long.xlsx
+++ b/processed_data_during_wm/processed_data_long.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="56">
   <si>
     <t>Team</t>
   </si>
@@ -543,7 +543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H330"/>
+  <dimension ref="A1:H385"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -7984,85 +7984,31 @@
     </row>
     <row r="287" spans="1:8">
       <c r="A287" t="s">
-        <v>9</v>
+        <v>55</v>
       </c>
       <c r="B287" s="2">
-        <v>46197</v>
-      </c>
-      <c r="C287">
-        <v>7</v>
-      </c>
-      <c r="D287">
-        <v>4.8743</v>
-      </c>
-      <c r="E287">
-        <v>0.173086</v>
-      </c>
-      <c r="F287">
-        <v>17.3086</v>
-      </c>
-      <c r="G287">
-        <v>0.185811</v>
-      </c>
-      <c r="H287">
-        <v>18.5811</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="288" spans="1:8">
       <c r="A288" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="B288" s="2">
-        <v>46197</v>
-      </c>
-      <c r="C288">
-        <v>7</v>
-      </c>
-      <c r="D288">
-        <v>6.4829</v>
-      </c>
-      <c r="E288">
-        <v>0.130139</v>
-      </c>
-      <c r="F288">
-        <v>13.0139</v>
-      </c>
-      <c r="G288">
-        <v>0.138911</v>
-      </c>
-      <c r="H288">
-        <v>13.8911</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="289" spans="1:8">
       <c r="A289" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="B289" s="2">
-        <v>46197</v>
-      </c>
-      <c r="C289">
-        <v>7</v>
-      </c>
-      <c r="D289">
-        <v>7.4514</v>
-      </c>
-      <c r="E289">
-        <v>0.113223</v>
-      </c>
-      <c r="F289">
-        <v>11.3223</v>
-      </c>
-      <c r="G289">
-        <v>0.120439</v>
-      </c>
-      <c r="H289">
-        <v>12.0439</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="290" spans="1:8">
       <c r="A290" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B290" s="2">
         <v>46197</v>
@@ -8071,24 +8017,24 @@
         <v>7</v>
       </c>
       <c r="D290">
-        <v>7.6071</v>
+        <v>4.8743</v>
       </c>
       <c r="E290">
-        <v>0.110905</v>
+        <v>0.173086</v>
       </c>
       <c r="F290">
-        <v>11.0905</v>
+        <v>17.3086</v>
       </c>
       <c r="G290">
-        <v>0.117909</v>
+        <v>0.185811</v>
       </c>
       <c r="H290">
-        <v>11.7909</v>
+        <v>18.5811</v>
       </c>
     </row>
     <row r="291" spans="1:8">
       <c r="A291" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B291" s="2">
         <v>46197</v>
@@ -8097,24 +8043,24 @@
         <v>7</v>
       </c>
       <c r="D291">
-        <v>10.8286</v>
+        <v>6.4829</v>
       </c>
       <c r="E291">
-        <v>0.077912</v>
+        <v>0.130139</v>
       </c>
       <c r="F291">
-        <v>7.7912</v>
+        <v>13.0139</v>
       </c>
       <c r="G291">
-        <v>0.081889</v>
+        <v>0.138911</v>
       </c>
       <c r="H291">
-        <v>8.1889</v>
+        <v>13.8911</v>
       </c>
     </row>
     <row r="292" spans="1:8">
       <c r="A292" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B292" s="2">
         <v>46197</v>
@@ -8123,24 +8069,24 @@
         <v>7</v>
       </c>
       <c r="D292">
-        <v>14.6</v>
+        <v>7.4514</v>
       </c>
       <c r="E292">
-        <v>0.057786</v>
+        <v>0.113223</v>
       </c>
       <c r="F292">
-        <v>5.7786</v>
+        <v>11.3223</v>
       </c>
       <c r="G292">
-        <v>0.059928</v>
+        <v>0.120439</v>
       </c>
       <c r="H292">
-        <v>5.9928</v>
+        <v>12.0439</v>
       </c>
     </row>
     <row r="293" spans="1:8">
       <c r="A293" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B293" s="2">
         <v>46197</v>
@@ -8149,24 +8095,24 @@
         <v>7</v>
       </c>
       <c r="D293">
-        <v>14.9429</v>
+        <v>7.6071</v>
       </c>
       <c r="E293">
-        <v>0.05646</v>
+        <v>0.110905</v>
       </c>
       <c r="F293">
-        <v>5.646</v>
+        <v>11.0905</v>
       </c>
       <c r="G293">
-        <v>0.058482</v>
+        <v>0.117909</v>
       </c>
       <c r="H293">
-        <v>5.8482</v>
+        <v>11.7909</v>
       </c>
     </row>
     <row r="294" spans="1:8">
       <c r="A294" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B294" s="2">
         <v>46197</v>
@@ -8175,24 +8121,24 @@
         <v>7</v>
       </c>
       <c r="D294">
-        <v>17.2286</v>
+        <v>10.8286</v>
       </c>
       <c r="E294">
-        <v>0.048969</v>
+        <v>0.077912</v>
       </c>
       <c r="F294">
-        <v>4.8969</v>
+        <v>7.7912</v>
       </c>
       <c r="G294">
-        <v>0.050314</v>
+        <v>0.081889</v>
       </c>
       <c r="H294">
-        <v>5.0314</v>
+        <v>8.1889</v>
       </c>
     </row>
     <row r="295" spans="1:8">
       <c r="A295" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B295" s="2">
         <v>46197</v>
@@ -8201,24 +8147,24 @@
         <v>7</v>
       </c>
       <c r="D295">
-        <v>32.1429</v>
+        <v>14.6</v>
       </c>
       <c r="E295">
-        <v>0.026248</v>
+        <v>0.057786</v>
       </c>
       <c r="F295">
-        <v>2.6248</v>
+        <v>5.7786</v>
       </c>
       <c r="G295">
-        <v>0.025582</v>
+        <v>0.059928</v>
       </c>
       <c r="H295">
-        <v>2.5582</v>
+        <v>5.9928</v>
       </c>
     </row>
     <row r="296" spans="1:8">
       <c r="A296" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B296" s="2">
         <v>46197</v>
@@ -8227,24 +8173,24 @@
         <v>7</v>
       </c>
       <c r="D296">
-        <v>32.4286</v>
+        <v>14.9429</v>
       </c>
       <c r="E296">
-        <v>0.026016</v>
+        <v>0.05646</v>
       </c>
       <c r="F296">
-        <v>2.6016</v>
+        <v>5.646</v>
       </c>
       <c r="G296">
-        <v>0.025331</v>
+        <v>0.058482</v>
       </c>
       <c r="H296">
-        <v>2.5331</v>
+        <v>5.8482</v>
       </c>
     </row>
     <row r="297" spans="1:8">
       <c r="A297" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B297" s="2">
         <v>46197</v>
@@ -8253,24 +8199,24 @@
         <v>7</v>
       </c>
       <c r="D297">
-        <v>35.1429</v>
+        <v>17.2286</v>
       </c>
       <c r="E297">
-        <v>0.024007</v>
+        <v>0.048969</v>
       </c>
       <c r="F297">
-        <v>2.4007</v>
+        <v>4.8969</v>
       </c>
       <c r="G297">
-        <v>0.023151</v>
+        <v>0.050314</v>
       </c>
       <c r="H297">
-        <v>2.3151</v>
+        <v>5.0314</v>
       </c>
     </row>
     <row r="298" spans="1:8">
       <c r="A298" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B298" s="2">
         <v>46197</v>
@@ -8279,24 +8225,24 @@
         <v>7</v>
       </c>
       <c r="D298">
-        <v>40</v>
+        <v>32.1429</v>
       </c>
       <c r="E298">
-        <v>0.021092</v>
+        <v>0.026248</v>
       </c>
       <c r="F298">
-        <v>2.1092</v>
+        <v>2.6248</v>
       </c>
       <c r="G298">
-        <v>0.019995</v>
+        <v>0.025582</v>
       </c>
       <c r="H298">
-        <v>1.9995</v>
+        <v>2.5582</v>
       </c>
     </row>
     <row r="299" spans="1:8">
       <c r="A299" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B299" s="2">
         <v>46197</v>
@@ -8305,24 +8251,24 @@
         <v>7</v>
       </c>
       <c r="D299">
-        <v>47</v>
+        <v>32.4286</v>
       </c>
       <c r="E299">
-        <v>0.01795</v>
+        <v>0.026016</v>
       </c>
       <c r="F299">
-        <v>1.795</v>
+        <v>2.6016</v>
       </c>
       <c r="G299">
-        <v>0.016604</v>
+        <v>0.025331</v>
       </c>
       <c r="H299">
-        <v>1.6604</v>
+        <v>2.5331</v>
       </c>
     </row>
     <row r="300" spans="1:8">
       <c r="A300" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B300" s="2">
         <v>46197</v>
@@ -8331,24 +8277,24 @@
         <v>7</v>
       </c>
       <c r="D300">
-        <v>52.5714</v>
+        <v>35.1429</v>
       </c>
       <c r="E300">
-        <v>0.016048</v>
+        <v>0.024007</v>
       </c>
       <c r="F300">
-        <v>1.6048</v>
+        <v>2.4007</v>
       </c>
       <c r="G300">
-        <v>0.014558</v>
+        <v>0.023151</v>
       </c>
       <c r="H300">
-        <v>1.4558</v>
+        <v>2.3151</v>
       </c>
     </row>
     <row r="301" spans="1:8">
       <c r="A301" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B301" s="2">
         <v>46197</v>
@@ -8357,24 +8303,24 @@
         <v>7</v>
       </c>
       <c r="D301">
-        <v>52.7143</v>
+        <v>40</v>
       </c>
       <c r="E301">
-        <v>0.016005</v>
+        <v>0.021092</v>
       </c>
       <c r="F301">
-        <v>1.6005</v>
+        <v>2.1092</v>
       </c>
       <c r="G301">
-        <v>0.014511</v>
+        <v>0.019995</v>
       </c>
       <c r="H301">
-        <v>1.4511</v>
+        <v>1.9995</v>
       </c>
     </row>
     <row r="302" spans="1:8">
       <c r="A302" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B302" s="2">
         <v>46197</v>
@@ -8383,24 +8329,24 @@
         <v>7</v>
       </c>
       <c r="D302">
-        <v>80.1429</v>
+        <v>47</v>
       </c>
       <c r="E302">
-        <v>0.010527</v>
+        <v>0.01795</v>
       </c>
       <c r="F302">
-        <v>1.0527</v>
+        <v>1.795</v>
       </c>
       <c r="G302">
-        <v>0.008680999999999999</v>
+        <v>0.016604</v>
       </c>
       <c r="H302">
-        <v>0.8681</v>
+        <v>1.6604</v>
       </c>
     </row>
     <row r="303" spans="1:8">
       <c r="A303" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B303" s="2">
         <v>46197</v>
@@ -8409,24 +8355,24 @@
         <v>7</v>
       </c>
       <c r="D303">
-        <v>112.2857</v>
+        <v>52.5714</v>
       </c>
       <c r="E303">
-        <v>0.007514</v>
+        <v>0.016048</v>
       </c>
       <c r="F303">
-        <v>0.7514</v>
+        <v>1.6048</v>
       </c>
       <c r="G303">
-        <v>0.005562</v>
+        <v>0.014558</v>
       </c>
       <c r="H303">
-        <v>0.5562</v>
+        <v>1.4558</v>
       </c>
     </row>
     <row r="304" spans="1:8">
       <c r="A304" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="B304" s="2">
         <v>46197</v>
@@ -8435,24 +8381,24 @@
         <v>7</v>
       </c>
       <c r="D304">
-        <v>137.8571</v>
+        <v>52.7143</v>
       </c>
       <c r="E304">
-        <v>0.00612</v>
+        <v>0.016005</v>
       </c>
       <c r="F304">
-        <v>0.612</v>
+        <v>1.6005</v>
       </c>
       <c r="G304">
-        <v>0.004169</v>
+        <v>0.014511</v>
       </c>
       <c r="H304">
-        <v>0.4169</v>
+        <v>1.4511</v>
       </c>
     </row>
     <row r="305" spans="1:8">
       <c r="A305" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B305" s="2">
         <v>46197</v>
@@ -8461,24 +8407,24 @@
         <v>7</v>
       </c>
       <c r="D305">
-        <v>138.5714</v>
+        <v>80.1429</v>
       </c>
       <c r="E305">
-        <v>0.006088</v>
+        <v>0.010527</v>
       </c>
       <c r="F305">
-        <v>0.6088</v>
+        <v>1.0527</v>
       </c>
       <c r="G305">
-        <v>0.004138</v>
+        <v>0.008680999999999999</v>
       </c>
       <c r="H305">
-        <v>0.4138</v>
+        <v>0.8681</v>
       </c>
     </row>
     <row r="306" spans="1:8">
       <c r="A306" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B306" s="2">
         <v>46197</v>
@@ -8487,24 +8433,24 @@
         <v>7</v>
       </c>
       <c r="D306">
-        <v>153.5714</v>
+        <v>112.2857</v>
       </c>
       <c r="E306">
-        <v>0.005494</v>
+        <v>0.007514</v>
       </c>
       <c r="F306">
-        <v>0.5494</v>
+        <v>0.7514</v>
       </c>
       <c r="G306">
-        <v>0.003561</v>
+        <v>0.005562</v>
       </c>
       <c r="H306">
-        <v>0.3561</v>
+        <v>0.5562</v>
       </c>
     </row>
     <row r="307" spans="1:8">
       <c r="A307" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B307" s="2">
         <v>46197</v>
@@ -8513,24 +8459,24 @@
         <v>7</v>
       </c>
       <c r="D307">
-        <v>187.2857</v>
+        <v>137.8571</v>
       </c>
       <c r="E307">
-        <v>0.004505</v>
+        <v>0.00612</v>
       </c>
       <c r="F307">
-        <v>0.4505</v>
+        <v>0.612</v>
       </c>
       <c r="G307">
-        <v>0.002636</v>
+        <v>0.004169</v>
       </c>
       <c r="H307">
-        <v>0.2636</v>
+        <v>0.4169</v>
       </c>
     </row>
     <row r="308" spans="1:8">
       <c r="A308" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B308" s="2">
         <v>46197</v>
@@ -8539,24 +8485,24 @@
         <v>7</v>
       </c>
       <c r="D308">
-        <v>188.2857</v>
+        <v>138.5714</v>
       </c>
       <c r="E308">
-        <v>0.004481</v>
+        <v>0.006088</v>
       </c>
       <c r="F308">
-        <v>0.4481</v>
+        <v>0.6088</v>
       </c>
       <c r="G308">
-        <v>0.002614</v>
+        <v>0.004138</v>
       </c>
       <c r="H308">
-        <v>0.2614</v>
+        <v>0.4138</v>
       </c>
     </row>
     <row r="309" spans="1:8">
       <c r="A309" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B309" s="2">
         <v>46197</v>
@@ -8565,24 +8511,24 @@
         <v>7</v>
       </c>
       <c r="D309">
-        <v>190</v>
+        <v>153.5714</v>
       </c>
       <c r="E309">
-        <v>0.00444</v>
+        <v>0.005494</v>
       </c>
       <c r="F309">
-        <v>0.444</v>
+        <v>0.5494</v>
       </c>
       <c r="G309">
-        <v>0.002578</v>
+        <v>0.003561</v>
       </c>
       <c r="H309">
-        <v>0.2578</v>
+        <v>0.3561</v>
       </c>
     </row>
     <row r="310" spans="1:8">
       <c r="A310" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B310" s="2">
         <v>46197</v>
@@ -8591,24 +8537,24 @@
         <v>7</v>
       </c>
       <c r="D310">
-        <v>206.3333</v>
+        <v>187.2857</v>
       </c>
       <c r="E310">
-        <v>0.004089</v>
+        <v>0.004505</v>
       </c>
       <c r="F310">
-        <v>0.4089</v>
+        <v>0.4505</v>
       </c>
       <c r="G310">
-        <v>0.002264</v>
+        <v>0.002636</v>
       </c>
       <c r="H310">
-        <v>0.2264</v>
+        <v>0.2636</v>
       </c>
     </row>
     <row r="311" spans="1:8">
       <c r="A311" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="B311" s="2">
         <v>46197</v>
@@ -8617,24 +8563,24 @@
         <v>7</v>
       </c>
       <c r="D311">
-        <v>232.5714</v>
+        <v>188.2857</v>
       </c>
       <c r="E311">
-        <v>0.003628</v>
+        <v>0.004481</v>
       </c>
       <c r="F311">
-        <v>0.3628</v>
+        <v>0.4481</v>
       </c>
       <c r="G311">
-        <v>0.001866</v>
+        <v>0.002614</v>
       </c>
       <c r="H311">
-        <v>0.1866</v>
+        <v>0.2614</v>
       </c>
     </row>
     <row r="312" spans="1:8">
       <c r="A312" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="B312" s="2">
         <v>46197</v>
@@ -8643,24 +8589,24 @@
         <v>7</v>
       </c>
       <c r="D312">
-        <v>288</v>
+        <v>190</v>
       </c>
       <c r="E312">
-        <v>0.002929</v>
+        <v>0.00444</v>
       </c>
       <c r="F312">
-        <v>0.2929</v>
+        <v>0.444</v>
       </c>
       <c r="G312">
-        <v>0.001304</v>
+        <v>0.002578</v>
       </c>
       <c r="H312">
-        <v>0.1304</v>
+        <v>0.2578</v>
       </c>
     </row>
     <row r="313" spans="1:8">
       <c r="A313" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B313" s="2">
         <v>46197</v>
@@ -8669,24 +8615,24 @@
         <v>7</v>
       </c>
       <c r="D313">
-        <v>289.2857</v>
+        <v>206.3333</v>
       </c>
       <c r="E313">
-        <v>0.002916</v>
+        <v>0.004089</v>
       </c>
       <c r="F313">
-        <v>0.2916</v>
+        <v>0.4089</v>
       </c>
       <c r="G313">
-        <v>0.001294</v>
+        <v>0.002264</v>
       </c>
       <c r="H313">
-        <v>0.1294</v>
+        <v>0.2264</v>
       </c>
     </row>
     <row r="314" spans="1:8">
       <c r="A314" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="B314" s="2">
         <v>46197</v>
@@ -8695,24 +8641,24 @@
         <v>7</v>
       </c>
       <c r="D314">
-        <v>314.4286</v>
+        <v>232.5714</v>
       </c>
       <c r="E314">
-        <v>0.002683</v>
+        <v>0.003628</v>
       </c>
       <c r="F314">
-        <v>0.2683</v>
+        <v>0.3628</v>
       </c>
       <c r="G314">
-        <v>0.00112</v>
+        <v>0.001866</v>
       </c>
       <c r="H314">
-        <v>0.112</v>
+        <v>0.1866</v>
       </c>
     </row>
     <row r="315" spans="1:8">
       <c r="A315" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B315" s="2">
         <v>46197</v>
@@ -8721,24 +8667,24 @@
         <v>7</v>
       </c>
       <c r="D315">
-        <v>320.1429</v>
+        <v>288</v>
       </c>
       <c r="E315">
-        <v>0.002635</v>
+        <v>0.002929</v>
       </c>
       <c r="F315">
-        <v>0.2635</v>
+        <v>0.2929</v>
       </c>
       <c r="G315">
-        <v>0.001085</v>
+        <v>0.001304</v>
       </c>
       <c r="H315">
-        <v>0.1085</v>
+        <v>0.1304</v>
       </c>
     </row>
     <row r="316" spans="1:8">
       <c r="A316" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="B316" s="2">
         <v>46197</v>
@@ -8747,24 +8693,24 @@
         <v>7</v>
       </c>
       <c r="D316">
-        <v>331</v>
+        <v>289.2857</v>
       </c>
       <c r="E316">
-        <v>0.002549</v>
+        <v>0.002916</v>
       </c>
       <c r="F316">
-        <v>0.2549</v>
+        <v>0.2916</v>
       </c>
       <c r="G316">
-        <v>0.001024</v>
+        <v>0.001294</v>
       </c>
       <c r="H316">
-        <v>0.1024</v>
+        <v>0.1294</v>
       </c>
     </row>
     <row r="317" spans="1:8">
       <c r="A317" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B317" s="2">
         <v>46197</v>
@@ -8773,24 +8719,24 @@
         <v>7</v>
       </c>
       <c r="D317">
-        <v>529.5714</v>
+        <v>314.4286</v>
       </c>
       <c r="E317">
-        <v>0.001593</v>
+        <v>0.002683</v>
       </c>
       <c r="F317">
-        <v>0.1593</v>
+        <v>0.2683</v>
       </c>
       <c r="G317">
-        <v>0.000434</v>
+        <v>0.00112</v>
       </c>
       <c r="H317">
-        <v>0.0434</v>
+        <v>0.112</v>
       </c>
     </row>
     <row r="318" spans="1:8">
       <c r="A318" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B318" s="2">
         <v>46197</v>
@@ -8799,24 +8745,24 @@
         <v>7</v>
       </c>
       <c r="D318">
-        <v>547.8570999999999</v>
+        <v>320.1429</v>
       </c>
       <c r="E318">
-        <v>0.00154</v>
+        <v>0.002635</v>
       </c>
       <c r="F318">
-        <v>0.154</v>
+        <v>0.2635</v>
       </c>
       <c r="G318">
-        <v>0.000407</v>
+        <v>0.001085</v>
       </c>
       <c r="H318">
-        <v>0.0407</v>
+        <v>0.1085</v>
       </c>
     </row>
     <row r="319" spans="1:8">
       <c r="A319" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B319" s="2">
         <v>46197</v>
@@ -8825,24 +8771,24 @@
         <v>7</v>
       </c>
       <c r="D319">
-        <v>583.5714</v>
+        <v>331</v>
       </c>
       <c r="E319">
-        <v>0.001446</v>
+        <v>0.002549</v>
       </c>
       <c r="F319">
-        <v>0.1446</v>
+        <v>0.2549</v>
       </c>
       <c r="G319">
-        <v>0.000361</v>
+        <v>0.001024</v>
       </c>
       <c r="H319">
-        <v>0.0361</v>
+        <v>0.1024</v>
       </c>
     </row>
     <row r="320" spans="1:8">
       <c r="A320" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="B320" s="2">
         <v>46197</v>
@@ -8851,24 +8797,24 @@
         <v>7</v>
       </c>
       <c r="D320">
-        <v>647.8570999999999</v>
+        <v>529.5714</v>
       </c>
       <c r="E320">
-        <v>0.001302</v>
+        <v>0.001593</v>
       </c>
       <c r="F320">
-        <v>0.1302</v>
+        <v>0.1593</v>
       </c>
       <c r="G320">
-        <v>0.000296</v>
+        <v>0.000434</v>
       </c>
       <c r="H320">
-        <v>0.0296</v>
+        <v>0.0434</v>
       </c>
     </row>
     <row r="321" spans="1:8">
       <c r="A321" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B321" s="2">
         <v>46197</v>
@@ -8877,24 +8823,24 @@
         <v>7</v>
       </c>
       <c r="D321">
-        <v>647.8570999999999</v>
+        <v>547.8570999999999</v>
       </c>
       <c r="E321">
-        <v>0.001302</v>
+        <v>0.00154</v>
       </c>
       <c r="F321">
-        <v>0.1302</v>
+        <v>0.154</v>
       </c>
       <c r="G321">
-        <v>0.000296</v>
+        <v>0.000407</v>
       </c>
       <c r="H321">
-        <v>0.0296</v>
+        <v>0.0407</v>
       </c>
     </row>
     <row r="322" spans="1:8">
       <c r="A322" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="B322" s="2">
         <v>46197</v>
@@ -8903,24 +8849,24 @@
         <v>7</v>
       </c>
       <c r="D322">
-        <v>747.8570999999999</v>
+        <v>583.5714</v>
       </c>
       <c r="E322">
-        <v>0.001128</v>
+        <v>0.001446</v>
       </c>
       <c r="F322">
-        <v>0.1128</v>
+        <v>0.1446</v>
       </c>
       <c r="G322">
-        <v>0.000224</v>
+        <v>0.000361</v>
       </c>
       <c r="H322">
-        <v>0.0224</v>
+        <v>0.0361</v>
       </c>
     </row>
     <row r="323" spans="1:8">
       <c r="A323" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B323" s="2">
         <v>46197</v>
@@ -8929,24 +8875,24 @@
         <v>7</v>
       </c>
       <c r="D323">
-        <v>855</v>
+        <v>647.8570999999999</v>
       </c>
       <c r="E323">
-        <v>0.000987</v>
+        <v>0.001302</v>
       </c>
       <c r="F323">
-        <v>0.0987</v>
+        <v>0.1302</v>
       </c>
       <c r="G323">
-        <v>0.000173</v>
+        <v>0.000296</v>
       </c>
       <c r="H323">
-        <v>0.0173</v>
+        <v>0.0296</v>
       </c>
     </row>
     <row r="324" spans="1:8">
       <c r="A324" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="B324" s="2">
         <v>46197</v>
@@ -8955,24 +8901,24 @@
         <v>7</v>
       </c>
       <c r="D324">
-        <v>890.7143</v>
+        <v>647.8570999999999</v>
       </c>
       <c r="E324">
-        <v>0.000947</v>
+        <v>0.001302</v>
       </c>
       <c r="F324">
-        <v>0.09470000000000001</v>
+        <v>0.1302</v>
       </c>
       <c r="G324">
-        <v>0.00016</v>
+        <v>0.000296</v>
       </c>
       <c r="H324">
-        <v>0.016</v>
+        <v>0.0296</v>
       </c>
     </row>
     <row r="325" spans="1:8">
       <c r="A325" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B325" s="2">
         <v>46197</v>
@@ -8981,24 +8927,24 @@
         <v>7</v>
       </c>
       <c r="D325">
-        <v>1212.1429</v>
+        <v>747.8570999999999</v>
       </c>
       <c r="E325">
-        <v>0.000696</v>
+        <v>0.001128</v>
       </c>
       <c r="F325">
-        <v>0.0696</v>
+        <v>0.1128</v>
       </c>
       <c r="G325">
-        <v>8.7E-05</v>
+        <v>0.000224</v>
       </c>
       <c r="H325">
-        <v>0.008699999999999999</v>
+        <v>0.0224</v>
       </c>
     </row>
     <row r="326" spans="1:8">
       <c r="A326" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B326" s="2">
         <v>46197</v>
@@ -9007,24 +8953,24 @@
         <v>7</v>
       </c>
       <c r="D326">
-        <v>1247.8571</v>
+        <v>855</v>
       </c>
       <c r="E326">
-        <v>0.000676</v>
+        <v>0.000987</v>
       </c>
       <c r="F326">
-        <v>0.06759999999999999</v>
+        <v>0.0987</v>
       </c>
       <c r="G326">
-        <v>8.2E-05</v>
+        <v>0.000173</v>
       </c>
       <c r="H326">
-        <v>0.008200000000000001</v>
+        <v>0.0173</v>
       </c>
     </row>
     <row r="327" spans="1:8">
       <c r="A327" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B327" s="2">
         <v>46197</v>
@@ -9033,24 +8979,24 @@
         <v>7</v>
       </c>
       <c r="D327">
-        <v>1569.2857</v>
+        <v>890.7143</v>
       </c>
       <c r="E327">
-        <v>0.000538</v>
+        <v>0.000947</v>
       </c>
       <c r="F327">
-        <v>0.0538</v>
+        <v>0.09470000000000001</v>
       </c>
       <c r="G327">
-        <v>5.2E-05</v>
+        <v>0.00016</v>
       </c>
       <c r="H327">
-        <v>0.0052</v>
+        <v>0.016</v>
       </c>
     </row>
     <row r="328" spans="1:8">
       <c r="A328" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B328" s="2">
         <v>46197</v>
@@ -9059,24 +9005,24 @@
         <v>7</v>
       </c>
       <c r="D328">
-        <v>1664</v>
+        <v>1212.1429</v>
       </c>
       <c r="E328">
-        <v>0.000507</v>
+        <v>0.000696</v>
       </c>
       <c r="F328">
-        <v>0.0507</v>
+        <v>0.0696</v>
       </c>
       <c r="G328">
-        <v>4.7E-05</v>
+        <v>8.7E-05</v>
       </c>
       <c r="H328">
-        <v>0.0047</v>
+        <v>0.008699999999999999</v>
       </c>
     </row>
     <row r="329" spans="1:8">
       <c r="A329" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B329" s="2">
         <v>46197</v>
@@ -9085,24 +9031,24 @@
         <v>7</v>
       </c>
       <c r="D329">
-        <v>1855</v>
+        <v>1247.8571</v>
       </c>
       <c r="E329">
-        <v>0.000455</v>
+        <v>0.000676</v>
       </c>
       <c r="F329">
-        <v>0.0455</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="G329">
-        <v>3.7E-05</v>
+        <v>8.2E-05</v>
       </c>
       <c r="H329">
-        <v>0.0037</v>
+        <v>0.008200000000000001</v>
       </c>
     </row>
     <row r="330" spans="1:8">
       <c r="A330" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B330" s="2">
         <v>46197</v>
@@ -9111,19 +9057,1251 @@
         <v>7</v>
       </c>
       <c r="D330">
+        <v>1569.2857</v>
+      </c>
+      <c r="E330">
+        <v>0.000538</v>
+      </c>
+      <c r="F330">
+        <v>0.0538</v>
+      </c>
+      <c r="G330">
+        <v>5.2E-05</v>
+      </c>
+      <c r="H330">
+        <v>0.0052</v>
+      </c>
+    </row>
+    <row r="331" spans="1:8">
+      <c r="A331" t="s">
+        <v>50</v>
+      </c>
+      <c r="B331" s="2">
+        <v>46197</v>
+      </c>
+      <c r="C331">
+        <v>7</v>
+      </c>
+      <c r="D331">
+        <v>1664</v>
+      </c>
+      <c r="E331">
+        <v>0.000507</v>
+      </c>
+      <c r="F331">
+        <v>0.0507</v>
+      </c>
+      <c r="G331">
+        <v>4.7E-05</v>
+      </c>
+      <c r="H331">
+        <v>0.0047</v>
+      </c>
+    </row>
+    <row r="332" spans="1:8">
+      <c r="A332" t="s">
+        <v>54</v>
+      </c>
+      <c r="B332" s="2">
+        <v>46197</v>
+      </c>
+      <c r="C332">
+        <v>7</v>
+      </c>
+      <c r="D332">
+        <v>1855</v>
+      </c>
+      <c r="E332">
+        <v>0.000455</v>
+      </c>
+      <c r="F332">
+        <v>0.0455</v>
+      </c>
+      <c r="G332">
+        <v>3.7E-05</v>
+      </c>
+      <c r="H332">
+        <v>0.0037</v>
+      </c>
+    </row>
+    <row r="333" spans="1:8">
+      <c r="A333" t="s">
+        <v>47</v>
+      </c>
+      <c r="B333" s="2">
+        <v>46197</v>
+      </c>
+      <c r="C333">
+        <v>7</v>
+      </c>
+      <c r="D333">
         <v>1926.4286</v>
       </c>
-      <c r="E330">
+      <c r="E333">
         <v>0.000438</v>
       </c>
-      <c r="F330">
+      <c r="F333">
         <v>0.0438</v>
       </c>
-      <c r="G330">
+      <c r="G333">
         <v>3.5E-05</v>
       </c>
-      <c r="H330">
+      <c r="H333">
         <v>0.0035</v>
+      </c>
+    </row>
+    <row r="334" spans="1:8">
+      <c r="A334" t="s">
+        <v>55</v>
+      </c>
+      <c r="B334" s="2">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="335" spans="1:8">
+      <c r="A335" t="s">
+        <v>53</v>
+      </c>
+      <c r="B335" s="2">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="336" spans="1:8">
+      <c r="A336" t="s">
+        <v>43</v>
+      </c>
+      <c r="B336" s="2">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="337" spans="1:8">
+      <c r="A337" t="s">
+        <v>25</v>
+      </c>
+      <c r="B337" s="2">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="338" spans="1:8">
+      <c r="A338" t="s">
+        <v>9</v>
+      </c>
+      <c r="B338" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C338">
+        <v>7</v>
+      </c>
+      <c r="D338">
+        <v>4.9586</v>
+      </c>
+      <c r="E338">
+        <v>0.173373</v>
+      </c>
+      <c r="F338">
+        <v>17.3373</v>
+      </c>
+      <c r="G338">
+        <v>0.184618</v>
+      </c>
+      <c r="H338">
+        <v>18.4618</v>
+      </c>
+    </row>
+    <row r="339" spans="1:8">
+      <c r="A339" t="s">
+        <v>8</v>
+      </c>
+      <c r="B339" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C339">
+        <v>7</v>
+      </c>
+      <c r="D339">
+        <v>6.6257</v>
+      </c>
+      <c r="E339">
+        <v>0.12975</v>
+      </c>
+      <c r="F339">
+        <v>12.975</v>
+      </c>
+      <c r="G339">
+        <v>0.137438</v>
+      </c>
+      <c r="H339">
+        <v>13.7438</v>
+      </c>
+    </row>
+    <row r="340" spans="1:8">
+      <c r="A340" t="s">
+        <v>13</v>
+      </c>
+      <c r="B340" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C340">
+        <v>7</v>
+      </c>
+      <c r="D340">
+        <v>7.0386</v>
+      </c>
+      <c r="E340">
+        <v>0.122139</v>
+      </c>
+      <c r="F340">
+        <v>12.2139</v>
+      </c>
+      <c r="G340">
+        <v>0.129207</v>
+      </c>
+      <c r="H340">
+        <v>12.9207</v>
+      </c>
+    </row>
+    <row r="341" spans="1:8">
+      <c r="A341" t="s">
+        <v>10</v>
+      </c>
+      <c r="B341" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C341">
+        <v>7</v>
+      </c>
+      <c r="D341">
+        <v>8.4343</v>
+      </c>
+      <c r="E341">
+        <v>0.101927</v>
+      </c>
+      <c r="F341">
+        <v>10.1927</v>
+      </c>
+      <c r="G341">
+        <v>0.107351</v>
+      </c>
+      <c r="H341">
+        <v>10.7351</v>
+      </c>
+    </row>
+    <row r="342" spans="1:8">
+      <c r="A342" t="s">
+        <v>11</v>
+      </c>
+      <c r="B342" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C342">
+        <v>7</v>
+      </c>
+      <c r="D342">
+        <v>10.5429</v>
+      </c>
+      <c r="E342">
+        <v>0.081542</v>
+      </c>
+      <c r="F342">
+        <v>8.154199999999999</v>
+      </c>
+      <c r="G342">
+        <v>0.08531</v>
+      </c>
+      <c r="H342">
+        <v>8.531000000000001</v>
+      </c>
+    </row>
+    <row r="343" spans="1:8">
+      <c r="A343" t="s">
+        <v>12</v>
+      </c>
+      <c r="B343" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C343">
+        <v>7</v>
+      </c>
+      <c r="D343">
+        <v>13.3143</v>
+      </c>
+      <c r="E343">
+        <v>0.064569</v>
+      </c>
+      <c r="F343">
+        <v>6.4569</v>
+      </c>
+      <c r="G343">
+        <v>0.06696299999999999</v>
+      </c>
+      <c r="H343">
+        <v>6.6963</v>
+      </c>
+    </row>
+    <row r="344" spans="1:8">
+      <c r="A344" t="s">
+        <v>15</v>
+      </c>
+      <c r="B344" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C344">
+        <v>7</v>
+      </c>
+      <c r="D344">
+        <v>15.9571</v>
+      </c>
+      <c r="E344">
+        <v>0.053875</v>
+      </c>
+      <c r="F344">
+        <v>5.3875</v>
+      </c>
+      <c r="G344">
+        <v>0.055408</v>
+      </c>
+      <c r="H344">
+        <v>5.5408</v>
+      </c>
+    </row>
+    <row r="345" spans="1:8">
+      <c r="A345" t="s">
+        <v>14</v>
+      </c>
+      <c r="B345" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C345">
+        <v>7</v>
+      </c>
+      <c r="D345">
+        <v>17.8</v>
+      </c>
+      <c r="E345">
+        <v>0.048297</v>
+      </c>
+      <c r="F345">
+        <v>4.8297</v>
+      </c>
+      <c r="G345">
+        <v>0.049383</v>
+      </c>
+      <c r="H345">
+        <v>4.9383</v>
+      </c>
+    </row>
+    <row r="346" spans="1:8">
+      <c r="A346" t="s">
+        <v>21</v>
+      </c>
+      <c r="B346" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C346">
+        <v>7</v>
+      </c>
+      <c r="D346">
+        <v>28.2857</v>
+      </c>
+      <c r="E346">
+        <v>0.030393</v>
+      </c>
+      <c r="F346">
+        <v>3.0393</v>
+      </c>
+      <c r="G346">
+        <v>0.030065</v>
+      </c>
+      <c r="H346">
+        <v>3.0065</v>
+      </c>
+    </row>
+    <row r="347" spans="1:8">
+      <c r="A347" t="s">
+        <v>16</v>
+      </c>
+      <c r="B347" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C347">
+        <v>7</v>
+      </c>
+      <c r="D347">
+        <v>32.7143</v>
+      </c>
+      <c r="E347">
+        <v>0.026279</v>
+      </c>
+      <c r="F347">
+        <v>2.6279</v>
+      </c>
+      <c r="G347">
+        <v>0.025635</v>
+      </c>
+      <c r="H347">
+        <v>2.5635</v>
+      </c>
+    </row>
+    <row r="348" spans="1:8">
+      <c r="A348" t="s">
+        <v>19</v>
+      </c>
+      <c r="B348" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C348">
+        <v>7</v>
+      </c>
+      <c r="D348">
+        <v>43.1429</v>
+      </c>
+      <c r="E348">
+        <v>0.019926</v>
+      </c>
+      <c r="F348">
+        <v>1.9926</v>
+      </c>
+      <c r="G348">
+        <v>0.018812</v>
+      </c>
+      <c r="H348">
+        <v>1.8812</v>
+      </c>
+    </row>
+    <row r="349" spans="1:8">
+      <c r="A349" t="s">
+        <v>22</v>
+      </c>
+      <c r="B349" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C349">
+        <v>7</v>
+      </c>
+      <c r="D349">
+        <v>45.7143</v>
+      </c>
+      <c r="E349">
+        <v>0.018806</v>
+      </c>
+      <c r="F349">
+        <v>1.8806</v>
+      </c>
+      <c r="G349">
+        <v>0.017611</v>
+      </c>
+      <c r="H349">
+        <v>1.7611</v>
+      </c>
+    </row>
+    <row r="350" spans="1:8">
+      <c r="A350" t="s">
+        <v>20</v>
+      </c>
+      <c r="B350" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C350">
+        <v>7</v>
+      </c>
+      <c r="D350">
+        <v>49.8571</v>
+      </c>
+      <c r="E350">
+        <v>0.017243</v>
+      </c>
+      <c r="F350">
+        <v>1.7243</v>
+      </c>
+      <c r="G350">
+        <v>0.01594</v>
+      </c>
+      <c r="H350">
+        <v>1.594</v>
+      </c>
+    </row>
+    <row r="351" spans="1:8">
+      <c r="A351" t="s">
+        <v>18</v>
+      </c>
+      <c r="B351" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C351">
+        <v>7</v>
+      </c>
+      <c r="D351">
+        <v>53.4286</v>
+      </c>
+      <c r="E351">
+        <v>0.01609</v>
+      </c>
+      <c r="F351">
+        <v>1.609</v>
+      </c>
+      <c r="G351">
+        <v>0.014709</v>
+      </c>
+      <c r="H351">
+        <v>1.4709</v>
+      </c>
+    </row>
+    <row r="352" spans="1:8">
+      <c r="A352" t="s">
+        <v>17</v>
+      </c>
+      <c r="B352" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C352">
+        <v>7</v>
+      </c>
+      <c r="D352">
+        <v>54.1429</v>
+      </c>
+      <c r="E352">
+        <v>0.015878</v>
+      </c>
+      <c r="F352">
+        <v>1.5878</v>
+      </c>
+      <c r="G352">
+        <v>0.014483</v>
+      </c>
+      <c r="H352">
+        <v>1.4483</v>
+      </c>
+    </row>
+    <row r="353" spans="1:8">
+      <c r="A353" t="s">
+        <v>24</v>
+      </c>
+      <c r="B353" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C353">
+        <v>7</v>
+      </c>
+      <c r="D353">
+        <v>76.4286</v>
+      </c>
+      <c r="E353">
+        <v>0.011248</v>
+      </c>
+      <c r="F353">
+        <v>1.1248</v>
+      </c>
+      <c r="G353">
+        <v>0.009575</v>
+      </c>
+      <c r="H353">
+        <v>0.9575</v>
+      </c>
+    </row>
+    <row r="354" spans="1:8">
+      <c r="A354" t="s">
+        <v>27</v>
+      </c>
+      <c r="B354" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C354">
+        <v>7</v>
+      </c>
+      <c r="D354">
+        <v>123.8571</v>
+      </c>
+      <c r="E354">
+        <v>0.006941</v>
+      </c>
+      <c r="F354">
+        <v>0.6941000000000001</v>
+      </c>
+      <c r="G354">
+        <v>0.005121</v>
+      </c>
+      <c r="H354">
+        <v>0.5121</v>
+      </c>
+    </row>
+    <row r="355" spans="1:8">
+      <c r="A355" t="s">
+        <v>26</v>
+      </c>
+      <c r="B355" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C355">
+        <v>7</v>
+      </c>
+      <c r="D355">
+        <v>132.2857</v>
+      </c>
+      <c r="E355">
+        <v>0.006499</v>
+      </c>
+      <c r="F355">
+        <v>0.6499</v>
+      </c>
+      <c r="G355">
+        <v>0.004678</v>
+      </c>
+      <c r="H355">
+        <v>0.4678</v>
+      </c>
+    </row>
+    <row r="356" spans="1:8">
+      <c r="A356" t="s">
+        <v>34</v>
+      </c>
+      <c r="B356" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C356">
+        <v>7</v>
+      </c>
+      <c r="D356">
+        <v>150.5714</v>
+      </c>
+      <c r="E356">
+        <v>0.005709</v>
+      </c>
+      <c r="F356">
+        <v>0.5709</v>
+      </c>
+      <c r="G356">
+        <v>0.003899</v>
+      </c>
+      <c r="H356">
+        <v>0.3899</v>
+      </c>
+    </row>
+    <row r="357" spans="1:8">
+      <c r="A357" t="s">
+        <v>28</v>
+      </c>
+      <c r="B357" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C357">
+        <v>7</v>
+      </c>
+      <c r="D357">
+        <v>165.7143</v>
+      </c>
+      <c r="E357">
+        <v>0.005188</v>
+      </c>
+      <c r="F357">
+        <v>0.5188</v>
+      </c>
+      <c r="G357">
+        <v>0.003394</v>
+      </c>
+      <c r="H357">
+        <v>0.3394</v>
+      </c>
+    </row>
+    <row r="358" spans="1:8">
+      <c r="A358" t="s">
+        <v>31</v>
+      </c>
+      <c r="B358" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C358">
+        <v>7</v>
+      </c>
+      <c r="D358">
+        <v>180.5714</v>
+      </c>
+      <c r="E358">
+        <v>0.004761</v>
+      </c>
+      <c r="F358">
+        <v>0.4761</v>
+      </c>
+      <c r="G358">
+        <v>0.002989</v>
+      </c>
+      <c r="H358">
+        <v>0.2989</v>
+      </c>
+    </row>
+    <row r="359" spans="1:8">
+      <c r="A359" t="s">
+        <v>30</v>
+      </c>
+      <c r="B359" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C359">
+        <v>7</v>
+      </c>
+      <c r="D359">
+        <v>181.1429</v>
+      </c>
+      <c r="E359">
+        <v>0.004746</v>
+      </c>
+      <c r="F359">
+        <v>0.4746</v>
+      </c>
+      <c r="G359">
+        <v>0.002975</v>
+      </c>
+      <c r="H359">
+        <v>0.2975</v>
+      </c>
+    </row>
+    <row r="360" spans="1:8">
+      <c r="A360" t="s">
+        <v>40</v>
+      </c>
+      <c r="B360" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C360">
+        <v>7</v>
+      </c>
+      <c r="D360">
+        <v>199.8333</v>
+      </c>
+      <c r="E360">
+        <v>0.004302</v>
+      </c>
+      <c r="F360">
+        <v>0.4302</v>
+      </c>
+      <c r="G360">
+        <v>0.002563</v>
+      </c>
+      <c r="H360">
+        <v>0.2563</v>
+      </c>
+    </row>
+    <row r="361" spans="1:8">
+      <c r="A361" t="s">
+        <v>29</v>
+      </c>
+      <c r="B361" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C361">
+        <v>7</v>
+      </c>
+      <c r="D361">
+        <v>205.4286</v>
+      </c>
+      <c r="E361">
+        <v>0.004185</v>
+      </c>
+      <c r="F361">
+        <v>0.4185</v>
+      </c>
+      <c r="G361">
+        <v>0.002456</v>
+      </c>
+      <c r="H361">
+        <v>0.2456</v>
+      </c>
+    </row>
+    <row r="362" spans="1:8">
+      <c r="A362" t="s">
+        <v>23</v>
+      </c>
+      <c r="B362" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C362">
+        <v>7</v>
+      </c>
+      <c r="D362">
+        <v>216.5714</v>
+      </c>
+      <c r="E362">
+        <v>0.00397</v>
+      </c>
+      <c r="F362">
+        <v>0.397</v>
+      </c>
+      <c r="G362">
+        <v>0.002263</v>
+      </c>
+      <c r="H362">
+        <v>0.2263</v>
+      </c>
+    </row>
+    <row r="363" spans="1:8">
+      <c r="A363" t="s">
+        <v>36</v>
+      </c>
+      <c r="B363" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C363">
+        <v>7</v>
+      </c>
+      <c r="D363">
+        <v>260.7143</v>
+      </c>
+      <c r="E363">
+        <v>0.003297</v>
+      </c>
+      <c r="F363">
+        <v>0.3297</v>
+      </c>
+      <c r="G363">
+        <v>0.001681</v>
+      </c>
+      <c r="H363">
+        <v>0.1681</v>
+      </c>
+    </row>
+    <row r="364" spans="1:8">
+      <c r="A364" t="s">
+        <v>32</v>
+      </c>
+      <c r="B364" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C364">
+        <v>7</v>
+      </c>
+      <c r="D364">
+        <v>327.1429</v>
+      </c>
+      <c r="E364">
+        <v>0.002628</v>
+      </c>
+      <c r="F364">
+        <v>0.2628</v>
+      </c>
+      <c r="G364">
+        <v>0.001149</v>
+      </c>
+      <c r="H364">
+        <v>0.1149</v>
+      </c>
+    </row>
+    <row r="365" spans="1:8">
+      <c r="A365" t="s">
+        <v>41</v>
+      </c>
+      <c r="B365" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C365">
+        <v>7</v>
+      </c>
+      <c r="D365">
+        <v>337.7143</v>
+      </c>
+      <c r="E365">
+        <v>0.002546</v>
+      </c>
+      <c r="F365">
+        <v>0.2546</v>
+      </c>
+      <c r="G365">
+        <v>0.001087</v>
+      </c>
+      <c r="H365">
+        <v>0.1087</v>
+      </c>
+    </row>
+    <row r="366" spans="1:8">
+      <c r="A366" t="s">
+        <v>38</v>
+      </c>
+      <c r="B366" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C366">
+        <v>7</v>
+      </c>
+      <c r="D366">
+        <v>509.4286</v>
+      </c>
+      <c r="E366">
+        <v>0.001688</v>
+      </c>
+      <c r="F366">
+        <v>0.1688</v>
+      </c>
+      <c r="G366">
+        <v>0.00052</v>
+      </c>
+      <c r="H366">
+        <v>0.052</v>
+      </c>
+    </row>
+    <row r="367" spans="1:8">
+      <c r="A367" t="s">
+        <v>46</v>
+      </c>
+      <c r="B367" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C367">
+        <v>7</v>
+      </c>
+      <c r="D367">
+        <v>569.2857</v>
+      </c>
+      <c r="E367">
+        <v>0.00151</v>
+      </c>
+      <c r="F367">
+        <v>0.151</v>
+      </c>
+      <c r="G367">
+        <v>0.000423</v>
+      </c>
+      <c r="H367">
+        <v>0.0423</v>
+      </c>
+    </row>
+    <row r="368" spans="1:8">
+      <c r="A368" t="s">
+        <v>39</v>
+      </c>
+      <c r="B368" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C368">
+        <v>7</v>
+      </c>
+      <c r="D368">
+        <v>570</v>
+      </c>
+      <c r="E368">
+        <v>0.001508</v>
+      </c>
+      <c r="F368">
+        <v>0.1508</v>
+      </c>
+      <c r="G368">
+        <v>0.000422</v>
+      </c>
+      <c r="H368">
+        <v>0.0422</v>
+      </c>
+    </row>
+    <row r="369" spans="1:8">
+      <c r="A369" t="s">
+        <v>37</v>
+      </c>
+      <c r="B369" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C369">
+        <v>7</v>
+      </c>
+      <c r="D369">
+        <v>576.4286</v>
+      </c>
+      <c r="E369">
+        <v>0.001491</v>
+      </c>
+      <c r="F369">
+        <v>0.1491</v>
+      </c>
+      <c r="G369">
+        <v>0.000413</v>
+      </c>
+      <c r="H369">
+        <v>0.0413</v>
+      </c>
+    </row>
+    <row r="370" spans="1:8">
+      <c r="A370" t="s">
+        <v>44</v>
+      </c>
+      <c r="B370" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C370">
+        <v>7</v>
+      </c>
+      <c r="D370">
+        <v>647.8570999999999</v>
+      </c>
+      <c r="E370">
+        <v>0.001327</v>
+      </c>
+      <c r="F370">
+        <v>0.1327</v>
+      </c>
+      <c r="G370">
+        <v>0.000331</v>
+      </c>
+      <c r="H370">
+        <v>0.0331</v>
+      </c>
+    </row>
+    <row r="371" spans="1:8">
+      <c r="A371" t="s">
+        <v>42</v>
+      </c>
+      <c r="B371" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C371">
+        <v>7</v>
+      </c>
+      <c r="D371">
+        <v>647.8570999999999</v>
+      </c>
+      <c r="E371">
+        <v>0.001327</v>
+      </c>
+      <c r="F371">
+        <v>0.1327</v>
+      </c>
+      <c r="G371">
+        <v>0.000331</v>
+      </c>
+      <c r="H371">
+        <v>0.0331</v>
+      </c>
+    </row>
+    <row r="372" spans="1:8">
+      <c r="A372" t="s">
+        <v>52</v>
+      </c>
+      <c r="B372" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C372">
+        <v>7</v>
+      </c>
+      <c r="D372">
+        <v>783.5714</v>
+      </c>
+      <c r="E372">
+        <v>0.001097</v>
+      </c>
+      <c r="F372">
+        <v>0.1097</v>
+      </c>
+      <c r="G372">
+        <v>0.00023</v>
+      </c>
+      <c r="H372">
+        <v>0.023</v>
+      </c>
+    </row>
+    <row r="373" spans="1:8">
+      <c r="A373" t="s">
+        <v>45</v>
+      </c>
+      <c r="B373" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C373">
+        <v>7</v>
+      </c>
+      <c r="D373">
+        <v>855</v>
+      </c>
+      <c r="E373">
+        <v>0.001005</v>
+      </c>
+      <c r="F373">
+        <v>0.1005</v>
+      </c>
+      <c r="G373">
+        <v>0.000195</v>
+      </c>
+      <c r="H373">
+        <v>0.0195</v>
+      </c>
+    </row>
+    <row r="374" spans="1:8">
+      <c r="A374" t="s">
+        <v>49</v>
+      </c>
+      <c r="B374" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C374">
+        <v>7</v>
+      </c>
+      <c r="D374">
+        <v>926.4286</v>
+      </c>
+      <c r="E374">
+        <v>0.000928</v>
+      </c>
+      <c r="F374">
+        <v>0.09279999999999999</v>
+      </c>
+      <c r="G374">
+        <v>0.000166</v>
+      </c>
+      <c r="H374">
+        <v>0.0166</v>
+      </c>
+    </row>
+    <row r="375" spans="1:8">
+      <c r="A375" t="s">
+        <v>51</v>
+      </c>
+      <c r="B375" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C375">
+        <v>7</v>
+      </c>
+      <c r="D375">
+        <v>1355</v>
+      </c>
+      <c r="E375">
+        <v>0.000634</v>
+      </c>
+      <c r="F375">
+        <v>0.0634</v>
+      </c>
+      <c r="G375">
+        <v>7.9E-05</v>
+      </c>
+      <c r="H375">
+        <v>0.007900000000000001</v>
+      </c>
+    </row>
+    <row r="376" spans="1:8">
+      <c r="A376" t="s">
+        <v>33</v>
+      </c>
+      <c r="B376" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C376">
+        <v>7</v>
+      </c>
+      <c r="D376">
+        <v>1569.2857</v>
+      </c>
+      <c r="E376">
+        <v>0.000548</v>
+      </c>
+      <c r="F376">
+        <v>0.0548</v>
+      </c>
+      <c r="G376">
+        <v>5.9E-05</v>
+      </c>
+      <c r="H376">
+        <v>0.0059</v>
+      </c>
+    </row>
+    <row r="377" spans="1:8">
+      <c r="A377" t="s">
+        <v>54</v>
+      </c>
+      <c r="B377" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C377">
+        <v>7</v>
+      </c>
+      <c r="D377">
+        <v>2001</v>
+      </c>
+      <c r="E377">
+        <v>0.00043</v>
+      </c>
+      <c r="F377">
+        <v>0.043</v>
+      </c>
+      <c r="G377">
+        <v>3.6E-05</v>
+      </c>
+      <c r="H377">
+        <v>0.0036</v>
+      </c>
+    </row>
+    <row r="378" spans="1:8">
+      <c r="A378" t="s">
+        <v>48</v>
+      </c>
+      <c r="B378" s="2">
+        <v>46199</v>
+      </c>
+      <c r="C378">
+        <v>7</v>
+      </c>
+      <c r="D378">
+        <v>2140.7143</v>
+      </c>
+      <c r="E378">
+        <v>0.000402</v>
+      </c>
+      <c r="F378">
+        <v>0.0402</v>
+      </c>
+      <c r="G378">
+        <v>3.2E-05</v>
+      </c>
+      <c r="H378">
+        <v>0.0032</v>
+      </c>
+    </row>
+    <row r="379" spans="1:8">
+      <c r="A379" t="s">
+        <v>55</v>
+      </c>
+      <c r="B379" s="2">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="380" spans="1:8">
+      <c r="A380" t="s">
+        <v>53</v>
+      </c>
+      <c r="B380" s="2">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="381" spans="1:8">
+      <c r="A381" t="s">
+        <v>47</v>
+      </c>
+      <c r="B381" s="2">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="382" spans="1:8">
+      <c r="A382" t="s">
+        <v>50</v>
+      </c>
+      <c r="B382" s="2">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="383" spans="1:8">
+      <c r="A383" t="s">
+        <v>35</v>
+      </c>
+      <c r="B383" s="2">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="384" spans="1:8">
+      <c r="A384" t="s">
+        <v>43</v>
+      </c>
+      <c r="B384" s="2">
+        <v>46199</v>
+      </c>
+    </row>
+    <row r="385" spans="1:2">
+      <c r="A385" t="s">
+        <v>25</v>
+      </c>
+      <c r="B385" s="2">
+        <v>46199</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add single predictions for semi-finals and update predictions 14.07.2026
</commit_message>
<xml_diff>
--- a/processed_data_during_wm/processed_data_long.xlsx
+++ b/processed_data_during_wm/processed_data_long.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="56">
   <si>
     <t>Team</t>
   </si>
@@ -543,7 +543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H769"/>
+  <dimension ref="A1:H817"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -15852,12 +15852,468 @@
         <v>46215</v>
       </c>
     </row>
-    <row r="769" spans="1:2">
+    <row r="769" spans="1:8">
       <c r="A769" t="s">
         <v>30</v>
       </c>
       <c r="B769" s="2">
         <v>46215</v>
+      </c>
+    </row>
+    <row r="770" spans="1:8">
+      <c r="A770" t="s">
+        <v>9</v>
+      </c>
+      <c r="B770" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C770">
+        <v>6</v>
+      </c>
+      <c r="D770">
+        <v>2.4312</v>
+      </c>
+      <c r="E770">
+        <v>0.389318</v>
+      </c>
+      <c r="F770">
+        <v>38.9318</v>
+      </c>
+      <c r="G770">
+        <v>0.39449</v>
+      </c>
+      <c r="H770">
+        <v>39.449</v>
+      </c>
+    </row>
+    <row r="771" spans="1:8">
+      <c r="A771" t="s">
+        <v>8</v>
+      </c>
+      <c r="B771" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C771">
+        <v>6</v>
+      </c>
+      <c r="D771">
+        <v>4.3286</v>
+      </c>
+      <c r="E771">
+        <v>0.21867</v>
+      </c>
+      <c r="F771">
+        <v>21.867</v>
+      </c>
+      <c r="G771">
+        <v>0.217498</v>
+      </c>
+      <c r="H771">
+        <v>21.7498</v>
+      </c>
+    </row>
+    <row r="772" spans="1:8">
+      <c r="A772" t="s">
+        <v>10</v>
+      </c>
+      <c r="B772" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C772">
+        <v>6</v>
+      </c>
+      <c r="D772">
+        <v>4.3619</v>
+      </c>
+      <c r="E772">
+        <v>0.216999</v>
+      </c>
+      <c r="F772">
+        <v>21.6999</v>
+      </c>
+      <c r="G772">
+        <v>0.215765</v>
+      </c>
+      <c r="H772">
+        <v>21.5765</v>
+      </c>
+    </row>
+    <row r="773" spans="1:8">
+      <c r="A773" t="s">
+        <v>13</v>
+      </c>
+      <c r="B773" s="2">
+        <v>46217</v>
+      </c>
+      <c r="C773">
+        <v>6</v>
+      </c>
+      <c r="D773">
+        <v>5.4083</v>
+      </c>
+      <c r="E773">
+        <v>0.175013</v>
+      </c>
+      <c r="F773">
+        <v>17.5013</v>
+      </c>
+      <c r="G773">
+        <v>0.172247</v>
+      </c>
+      <c r="H773">
+        <v>17.2247</v>
+      </c>
+    </row>
+    <row r="774" spans="1:8">
+      <c r="A774" t="s">
+        <v>37</v>
+      </c>
+      <c r="B774" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="775" spans="1:8">
+      <c r="A775" t="s">
+        <v>40</v>
+      </c>
+      <c r="B775" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="776" spans="1:8">
+      <c r="A776" t="s">
+        <v>17</v>
+      </c>
+      <c r="B776" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="777" spans="1:8">
+      <c r="A777" t="s">
+        <v>38</v>
+      </c>
+      <c r="B777" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="778" spans="1:8">
+      <c r="A778" t="s">
+        <v>12</v>
+      </c>
+      <c r="B778" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="779" spans="1:8">
+      <c r="A779" t="s">
+        <v>54</v>
+      </c>
+      <c r="B779" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="780" spans="1:8">
+      <c r="A780" t="s">
+        <v>44</v>
+      </c>
+      <c r="B780" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="781" spans="1:8">
+      <c r="A781" t="s">
+        <v>14</v>
+      </c>
+      <c r="B781" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="782" spans="1:8">
+      <c r="A782" t="s">
+        <v>27</v>
+      </c>
+      <c r="B782" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="783" spans="1:8">
+      <c r="A783" t="s">
+        <v>34</v>
+      </c>
+      <c r="B783" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="784" spans="1:8">
+      <c r="A784" t="s">
+        <v>41</v>
+      </c>
+      <c r="B784" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="785" spans="1:2">
+      <c r="A785" t="s">
+        <v>55</v>
+      </c>
+      <c r="B785" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="786" spans="1:2">
+      <c r="A786" t="s">
+        <v>48</v>
+      </c>
+      <c r="B786" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="787" spans="1:2">
+      <c r="A787" t="s">
+        <v>42</v>
+      </c>
+      <c r="B787" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="788" spans="1:2">
+      <c r="A788" t="s">
+        <v>20</v>
+      </c>
+      <c r="B788" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="789" spans="1:2">
+      <c r="A789" t="s">
+        <v>53</v>
+      </c>
+      <c r="B789" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="790" spans="1:2">
+      <c r="A790" t="s">
+        <v>31</v>
+      </c>
+      <c r="B790" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="791" spans="1:2">
+      <c r="A791" t="s">
+        <v>52</v>
+      </c>
+      <c r="B791" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="792" spans="1:2">
+      <c r="A792" t="s">
+        <v>47</v>
+      </c>
+      <c r="B792" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="793" spans="1:2">
+      <c r="A793" t="s">
+        <v>18</v>
+      </c>
+      <c r="B793" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="794" spans="1:2">
+      <c r="A794" t="s">
+        <v>26</v>
+      </c>
+      <c r="B794" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="795" spans="1:2">
+      <c r="A795" t="s">
+        <v>19</v>
+      </c>
+      <c r="B795" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="796" spans="1:2">
+      <c r="A796" t="s">
+        <v>22</v>
+      </c>
+      <c r="B796" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="797" spans="1:2">
+      <c r="A797" t="s">
+        <v>49</v>
+      </c>
+      <c r="B797" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="798" spans="1:2">
+      <c r="A798" t="s">
+        <v>15</v>
+      </c>
+      <c r="B798" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="799" spans="1:2">
+      <c r="A799" t="s">
+        <v>16</v>
+      </c>
+      <c r="B799" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="800" spans="1:2">
+      <c r="A800" t="s">
+        <v>50</v>
+      </c>
+      <c r="B800" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="801" spans="1:2">
+      <c r="A801" t="s">
+        <v>32</v>
+      </c>
+      <c r="B801" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="802" spans="1:2">
+      <c r="A802" t="s">
+        <v>11</v>
+      </c>
+      <c r="B802" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="803" spans="1:2">
+      <c r="A803" t="s">
+        <v>45</v>
+      </c>
+      <c r="B803" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="804" spans="1:2">
+      <c r="A804" t="s">
+        <v>33</v>
+      </c>
+      <c r="B804" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="805" spans="1:2">
+      <c r="A805" t="s">
+        <v>29</v>
+      </c>
+      <c r="B805" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="806" spans="1:2">
+      <c r="A806" t="s">
+        <v>24</v>
+      </c>
+      <c r="B806" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="807" spans="1:2">
+      <c r="A807" t="s">
+        <v>28</v>
+      </c>
+      <c r="B807" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="808" spans="1:2">
+      <c r="A808" t="s">
+        <v>46</v>
+      </c>
+      <c r="B808" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="809" spans="1:2">
+      <c r="A809" t="s">
+        <v>39</v>
+      </c>
+      <c r="B809" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="810" spans="1:2">
+      <c r="A810" t="s">
+        <v>35</v>
+      </c>
+      <c r="B810" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="811" spans="1:2">
+      <c r="A811" t="s">
+        <v>43</v>
+      </c>
+      <c r="B811" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="812" spans="1:2">
+      <c r="A812" t="s">
+        <v>25</v>
+      </c>
+      <c r="B812" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="813" spans="1:2">
+      <c r="A813" t="s">
+        <v>21</v>
+      </c>
+      <c r="B813" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="814" spans="1:2">
+      <c r="A814" t="s">
+        <v>23</v>
+      </c>
+      <c r="B814" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="815" spans="1:2">
+      <c r="A815" t="s">
+        <v>51</v>
+      </c>
+      <c r="B815" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="816" spans="1:2">
+      <c r="A816" t="s">
+        <v>36</v>
+      </c>
+      <c r="B816" s="2">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="817" spans="1:2">
+      <c r="A817" t="s">
+        <v>30</v>
+      </c>
+      <c r="B817" s="2">
+        <v>46217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add single match predictions and update final prediction 16.07.2026
</commit_message>
<xml_diff>
--- a/processed_data_during_wm/processed_data_long.xlsx
+++ b/processed_data_during_wm/processed_data_long.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="824" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="56">
   <si>
     <t>Team</t>
   </si>
@@ -543,7 +543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H817"/>
+  <dimension ref="A1:H865"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -16308,12 +16308,432 @@
         <v>46217</v>
       </c>
     </row>
-    <row r="817" spans="1:2">
+    <row r="817" spans="1:8">
       <c r="A817" t="s">
         <v>30</v>
       </c>
       <c r="B817" s="2">
         <v>46217</v>
+      </c>
+    </row>
+    <row r="818" spans="1:8">
+      <c r="A818" t="s">
+        <v>8</v>
+      </c>
+      <c r="B818" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C818">
+        <v>6</v>
+      </c>
+      <c r="D818">
+        <v>1.6396</v>
+      </c>
+      <c r="E818">
+        <v>0.5806249999999999</v>
+      </c>
+      <c r="F818">
+        <v>58.0625</v>
+      </c>
+      <c r="G818">
+        <v>0.584691</v>
+      </c>
+      <c r="H818">
+        <v>58.4691</v>
+      </c>
+    </row>
+    <row r="819" spans="1:8">
+      <c r="A819" t="s">
+        <v>13</v>
+      </c>
+      <c r="B819" s="2">
+        <v>46219</v>
+      </c>
+      <c r="C819">
+        <v>6</v>
+      </c>
+      <c r="D819">
+        <v>2.27</v>
+      </c>
+      <c r="E819">
+        <v>0.419375</v>
+      </c>
+      <c r="F819">
+        <v>41.9375</v>
+      </c>
+      <c r="G819">
+        <v>0.415309</v>
+      </c>
+      <c r="H819">
+        <v>41.5309</v>
+      </c>
+    </row>
+    <row r="820" spans="1:8">
+      <c r="A820" t="s">
+        <v>37</v>
+      </c>
+      <c r="B820" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="821" spans="1:8">
+      <c r="A821" t="s">
+        <v>40</v>
+      </c>
+      <c r="B821" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="822" spans="1:8">
+      <c r="A822" t="s">
+        <v>17</v>
+      </c>
+      <c r="B822" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="823" spans="1:8">
+      <c r="A823" t="s">
+        <v>38</v>
+      </c>
+      <c r="B823" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="824" spans="1:8">
+      <c r="A824" t="s">
+        <v>12</v>
+      </c>
+      <c r="B824" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="825" spans="1:8">
+      <c r="A825" t="s">
+        <v>54</v>
+      </c>
+      <c r="B825" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="826" spans="1:8">
+      <c r="A826" t="s">
+        <v>44</v>
+      </c>
+      <c r="B826" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="827" spans="1:8">
+      <c r="A827" t="s">
+        <v>14</v>
+      </c>
+      <c r="B827" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="828" spans="1:8">
+      <c r="A828" t="s">
+        <v>27</v>
+      </c>
+      <c r="B828" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="829" spans="1:8">
+      <c r="A829" t="s">
+        <v>34</v>
+      </c>
+      <c r="B829" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="830" spans="1:8">
+      <c r="A830" t="s">
+        <v>10</v>
+      </c>
+      <c r="B830" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="831" spans="1:8">
+      <c r="A831" t="s">
+        <v>9</v>
+      </c>
+      <c r="B831" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="832" spans="1:8">
+      <c r="A832" t="s">
+        <v>41</v>
+      </c>
+      <c r="B832" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="833" spans="1:2">
+      <c r="A833" t="s">
+        <v>55</v>
+      </c>
+      <c r="B833" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="834" spans="1:2">
+      <c r="A834" t="s">
+        <v>48</v>
+      </c>
+      <c r="B834" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="835" spans="1:2">
+      <c r="A835" t="s">
+        <v>42</v>
+      </c>
+      <c r="B835" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="836" spans="1:2">
+      <c r="A836" t="s">
+        <v>20</v>
+      </c>
+      <c r="B836" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="837" spans="1:2">
+      <c r="A837" t="s">
+        <v>53</v>
+      </c>
+      <c r="B837" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="838" spans="1:2">
+      <c r="A838" t="s">
+        <v>31</v>
+      </c>
+      <c r="B838" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="839" spans="1:2">
+      <c r="A839" t="s">
+        <v>52</v>
+      </c>
+      <c r="B839" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="840" spans="1:2">
+      <c r="A840" t="s">
+        <v>47</v>
+      </c>
+      <c r="B840" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="841" spans="1:2">
+      <c r="A841" t="s">
+        <v>18</v>
+      </c>
+      <c r="B841" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="842" spans="1:2">
+      <c r="A842" t="s">
+        <v>26</v>
+      </c>
+      <c r="B842" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="843" spans="1:2">
+      <c r="A843" t="s">
+        <v>19</v>
+      </c>
+      <c r="B843" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="844" spans="1:2">
+      <c r="A844" t="s">
+        <v>22</v>
+      </c>
+      <c r="B844" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="845" spans="1:2">
+      <c r="A845" t="s">
+        <v>49</v>
+      </c>
+      <c r="B845" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="846" spans="1:2">
+      <c r="A846" t="s">
+        <v>15</v>
+      </c>
+      <c r="B846" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="847" spans="1:2">
+      <c r="A847" t="s">
+        <v>16</v>
+      </c>
+      <c r="B847" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="848" spans="1:2">
+      <c r="A848" t="s">
+        <v>50</v>
+      </c>
+      <c r="B848" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="849" spans="1:2">
+      <c r="A849" t="s">
+        <v>32</v>
+      </c>
+      <c r="B849" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="850" spans="1:2">
+      <c r="A850" t="s">
+        <v>11</v>
+      </c>
+      <c r="B850" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="851" spans="1:2">
+      <c r="A851" t="s">
+        <v>45</v>
+      </c>
+      <c r="B851" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="852" spans="1:2">
+      <c r="A852" t="s">
+        <v>33</v>
+      </c>
+      <c r="B852" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="853" spans="1:2">
+      <c r="A853" t="s">
+        <v>29</v>
+      </c>
+      <c r="B853" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="854" spans="1:2">
+      <c r="A854" t="s">
+        <v>24</v>
+      </c>
+      <c r="B854" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="855" spans="1:2">
+      <c r="A855" t="s">
+        <v>28</v>
+      </c>
+      <c r="B855" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="856" spans="1:2">
+      <c r="A856" t="s">
+        <v>46</v>
+      </c>
+      <c r="B856" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="857" spans="1:2">
+      <c r="A857" t="s">
+        <v>39</v>
+      </c>
+      <c r="B857" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="858" spans="1:2">
+      <c r="A858" t="s">
+        <v>35</v>
+      </c>
+      <c r="B858" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="859" spans="1:2">
+      <c r="A859" t="s">
+        <v>43</v>
+      </c>
+      <c r="B859" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="860" spans="1:2">
+      <c r="A860" t="s">
+        <v>25</v>
+      </c>
+      <c r="B860" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="861" spans="1:2">
+      <c r="A861" t="s">
+        <v>21</v>
+      </c>
+      <c r="B861" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="862" spans="1:2">
+      <c r="A862" t="s">
+        <v>23</v>
+      </c>
+      <c r="B862" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="863" spans="1:2">
+      <c r="A863" t="s">
+        <v>51</v>
+      </c>
+      <c r="B863" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="864" spans="1:2">
+      <c r="A864" t="s">
+        <v>36</v>
+      </c>
+      <c r="B864" s="2">
+        <v>46219</v>
+      </c>
+    </row>
+    <row r="865" spans="1:2">
+      <c r="A865" t="s">
+        <v>30</v>
+      </c>
+      <c r="B865" s="2">
+        <v>46219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>